<commit_message>
feat: add volleyball C-class tests T16-T19
</commit_message>
<xml_diff>
--- a/docs/scoring-sheet.xlsx
+++ b/docs/scoring-sheet.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,8 +161,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -528,11 +526,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -545,14 +543,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>长基线双目系统标定测试打分表（LBST-TEST-001）</t>
+          <t>27RC 排球机器人视觉系统测试打分表（27RC-VBT-001）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>填写说明：单项得分只填 100 / 80 / 60 / 0 或 N/A；B 类可填 N/A（自动剔除权重并归一化），A 类（T01–T10）不允许 N/A；打分依据见 docs/test-procedures.md。</t>
+          <t>填写说明：单项得分只填 100 / 80 / 60 / 0 或 N/A；B 类可填 N/A（自动剔除权重并归一化），A 类（T01–T10）与 C 类（T16–T19）不允许 N/A；权重分布 A 50 / B 20 / C 30；打分依据见 docs/test-procedures.md。</t>
         </is>
       </c>
     </row>
@@ -620,7 +618,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="4">
@@ -654,7 +652,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="4">
@@ -688,7 +686,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="4">
@@ -722,7 +720,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="4">
@@ -756,7 +754,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="4">
@@ -790,7 +788,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="4">
@@ -824,7 +822,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="4">
@@ -858,7 +856,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="4">
@@ -892,7 +890,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="4">
@@ -926,7 +924,7 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="4">
@@ -960,7 +958,7 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="4">
@@ -994,7 +992,7 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="4">
@@ -1028,7 +1026,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="4">
@@ -1062,7 +1060,7 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="4">
@@ -1096,7 +1094,7 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="4">
@@ -1114,63 +1112,199 @@
       <c r="I18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>排球检测模型精度</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="4">
+        <f>IF(ISNUMBER(E19),D19*E19/100,0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
+        <f>IF(ISNUMBER(E19),D19,0)</f>
+        <v/>
+      </c>
+      <c r="H19" s="4">
+        <f>IF(NOT(ISNUMBER(E19)),"N/A",IF(E19&gt;=100,"优",IF(E19&gt;=80,"良",IF(E19&gt;=60,"合格","不合格"))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>检测推理速度</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="4">
+        <f>IF(ISNUMBER(E20),D20*E20/100,0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="4">
+        <f>IF(ISNUMBER(E20),D20,0)</f>
+        <v/>
+      </c>
+      <c r="H20" s="4">
+        <f>IF(NOT(ISNUMBER(E20)),"N/A",IF(E20&gt;=100,"优",IF(E20&gt;=80,"良",IF(E20&gt;=60,"合格","不合格"))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>动态球测距</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="4">
+        <f>IF(ISNUMBER(E21),D21*E21/100,0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="4">
+        <f>IF(ISNUMBER(E21),D21,0)</f>
+        <v/>
+      </c>
+      <c r="H21" s="4">
+        <f>IF(NOT(ISNUMBER(E21)),"N/A",IF(E21&gt;=100,"优",IF(E21&gt;=80,"良",IF(E21&gt;=60,"合格","不合格"))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>发球时机与自动击球闭环</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="4">
+        <f>IF(ISNUMBER(E22),D22*E22/100,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="4">
+        <f>IF(ISNUMBER(E22),D22,0)</f>
+        <v/>
+      </c>
+      <c r="H22" s="4">
+        <f>IF(NOT(ISNUMBER(E22)),"N/A",IF(E22&gt;=100,"优",IF(E22&gt;=80,"良",IF(E22&gt;=60,"合格","不合格"))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="7">
-        <f>SUM(D4:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="7">
-        <f>SUM(F4:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="7">
-        <f>SUM(G4:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="9" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>合计（A 50 / B 20 / C 30）</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="7">
+        <f>SUM(D4:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="7">
+        <f>SUM(F4:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="7">
+        <f>SUM(G4:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>总分 S</t>
         </is>
       </c>
-      <c r="B21" s="11">
-        <f>IF(SUM(G4:G18)=0,"",ROUND(SUM(F4:F18)/SUM(G4:G18)*100,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="B25" s="11">
+        <f>IF(SUM(G4:G22)=0,"",ROUND(SUM(F4:F22)/SUM(G4:G22)*100,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>否决项触发（联动否决项检查表）</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B26" s="11">
         <f>IF(COUNTIF('否决项检查'!C3:C6,"是")&gt;0,"是","否")</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>等级（A/B/C/F）</t>
         </is>
       </c>
-      <c r="B23" s="12">
-        <f>IF(B22="是","F",IF(NOT(ISNUMBER(B21)),"",IF(AND(B21&gt;=90,COUNT(E4:E13)=10),"A",IF(B21&gt;=80,"B",IF(AND(B21&gt;=70,COUNTIF(E4:E13,0)=0),"C","F")))))</f>
+      <c r="B27" s="12">
+        <f>IF(B26="是","F",IF(NOT(ISNUMBER(B25)),"",IF(AND(B25&gt;=90,COUNT(E4:E13)=10),"A",IF(B25&gt;=80,"B",IF(AND(B25&gt;=70,COUNTIF(E4:E13,0)=0),"C","F")))))</f>
         <v/>
       </c>
     </row>
@@ -1180,7 +1314,7 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="单项得分" prompt="填写 100 / 80 / 60 / 0；B 类可填 N/A" type="list">
+    <dataValidation sqref="E4:E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="单项得分" prompt="填写 100 / 80 / 60 / 0；B 类可填 N/A" type="list">
       <formula1>"100,80,60,0,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1360,7 +1494,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>'打分汇总'!B21</f>
+        <f>'打分汇总'!B25</f>
         <v/>
       </c>
     </row>
@@ -1371,7 +1505,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>'打分汇总'!B23</f>
+        <f>'打分汇总'!B27</f>
         <v/>
       </c>
     </row>
@@ -1383,7 +1517,7 @@
       </c>
       <c r="B8" s="5" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>主要问题与建议</t>
@@ -1397,15 +1531,15 @@
           <t>签字 / 日期</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
+      <c r="B10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
-      <c r="B11" s="13" t="n"/>
+      <c r="B11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
-      <c r="B12" s="14" t="n"/>
+      <c r="B12" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>